<commit_message>
data: publish 2026-10-21 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-21-182路.xlsx
+++ b/data/export/2026-10-21-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -743,32 +743,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +780,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,17 +804,17 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -820,13 +824,17 @@
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -887,7 +895,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -926,7 +934,7 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
@@ -937,7 +945,7 @@
       <c r="AB4" s="2" t="inlineStr"/>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -998,7 +1006,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1037,7 +1045,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1048,7 +1056,7 @@
       <c r="AB5" s="2" t="inlineStr"/>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1076,32 +1084,36 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:56</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1109,7 +1121,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1133,17 +1145,17 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z6" s="2" t="inlineStr">
@@ -1153,13 +1165,17 @@
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB6" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB6" s="2" t="inlineStr">
+        <is>
+          <t>81.0</t>
+        </is>
+      </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1236,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1270,7 +1286,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1347,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1397,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1442,7 +1458,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1492,7 +1508,7 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
         </is>
       </c>
     </row>
@@ -1500,22 +1516,22 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>沪A35717D</t>
+          <t>沪A67353D</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1548,12 +1564,12 @@
       <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:42</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1567,7 +1583,7 @@
       <c r="T10" s="2" t="inlineStr"/>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>07:12</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
@@ -1603,7 +1619,784 @@
       <c r="AB10" s="2" t="inlineStr"/>
       <c r="AC10" s="2" t="inlineStr">
         <is>
-          <t>—/9</t>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr"/>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr"/>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr"/>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:22</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr"/>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>—/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-21 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-21-182路.xlsx
+++ b/data/export/2026-10-21-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC24"/>
+  <dimension ref="A1:AC25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -899,7 +899,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1256,7 +1256,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1449,32 +1449,36 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>94分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
           <t>06:22</t>
@@ -1482,7 +1486,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1506,17 +1510,17 @@
       </c>
       <c r="W9" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z9" s="2" t="inlineStr">
@@ -1526,13 +1530,17 @@
       </c>
       <c r="AA9" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB9" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>94.0</t>
+        </is>
+      </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1601,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1632,7 +1640,7 @@
       </c>
       <c r="Z10" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA10" s="2" t="inlineStr">
@@ -1704,7 +1712,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1815,7 +1823,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1926,7 +1934,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2037,7 +2045,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2148,7 +2156,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2259,7 +2267,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2374,7 +2382,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2489,7 +2497,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2604,7 +2612,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>08:12</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2830,7 +2838,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2884,7 +2892,7 @@
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2945,7 +2953,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3056,7 +3064,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -3100,13 +3108,17 @@
       </c>
       <c r="AA23" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB23" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB23" s="2" t="inlineStr">
+        <is>
+          <t>94.0</t>
+        </is>
+      </c>
       <c r="AC23" s="2" t="inlineStr">
         <is>
-          <t>—/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -3167,7 +3179,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:32</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3221,6 +3233,117 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>06:42</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB25" s="2" t="inlineStr"/>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>—/14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>